<commit_message>
update sprint 6 metrics
</commit_message>
<xml_diff>
--- a/sprint6/26-04-6-metrics.xlsx
+++ b/sprint6/26-04-6-metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\styne\Lewis\1-Spring26\software\sprint6\Stone-Ocean-Backlogs\sprint6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D36B4ECE-EA42-4050-992C-4D686FE3E428}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD9522E5-F452-4706-9394-8F6FA6F2CAB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="43">
   <si>
     <t>Name</t>
   </si>
@@ -164,6 +164,12 @@
   </si>
   <si>
     <t>April 14th, 2026; 9:55am</t>
+  </si>
+  <si>
+    <t>RW</t>
+  </si>
+  <si>
+    <t>April 14th, 2026; 10:10am</t>
   </si>
 </sst>
 </file>
@@ -37138,7 +37144,7 @@
       </c>
       <c r="F9" s="8"/>
       <c r="G9" s="9">
-        <f t="shared" ref="G9:H14" si="0">D9/B9</f>
+        <f t="shared" ref="G9:H12" si="0">D9/B9</f>
         <v>0</v>
       </c>
       <c r="H9" s="10" t="e">
@@ -37349,9 +37355,13 @@
       <c r="A21" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B21" s="10"/>
+      <c r="B21" s="10" t="s">
+        <v>41</v>
+      </c>
       <c r="C21" s="16"/>
-      <c r="D21" s="17"/>
+      <c r="D21" s="17" t="s">
+        <v>42</v>
+      </c>
       <c r="E21" s="7"/>
     </row>
     <row r="22" spans="1:9" ht="15.75" customHeight="1">

</xml_diff>

<commit_message>
Update the Sprint6 backlogs, update sprint6 metrics, create sprint6 initial metrics
</commit_message>
<xml_diff>
--- a/sprint6/26-04-6-metrics.xlsx
+++ b/sprint6/26-04-6-metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\styne\Lewis\1-Spring26\software\sprint6\Stone-Ocean-Backlogs\sprint6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD9522E5-F452-4706-9394-8F6FA6F2CAB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13000CD2-F357-445C-945B-6CA818C6AAC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9876" yWindow="1128" windowWidth="11472" windowHeight="10776" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Example" sheetId="8" r:id="rId1"/>
@@ -37134,7 +37134,7 @@
         <v>6</v>
       </c>
       <c r="C9" s="7">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D9" s="7">
         <v>0</v>
@@ -37147,9 +37147,9 @@
         <f t="shared" ref="G9:H12" si="0">D9/B9</f>
         <v>0</v>
       </c>
-      <c r="H9" s="10" t="e">
+      <c r="H9" s="10">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="I9" s="10">
         <f t="shared" ref="I9:I16" si="1">E9/B9</f>
@@ -37164,7 +37164,7 @@
         <v>6</v>
       </c>
       <c r="C10" s="7">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D10" s="7">
         <v>0</v>
@@ -37177,9 +37177,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H10" s="10" t="e">
+      <c r="H10" s="10">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="I10" s="10">
         <f t="shared" si="1"/>
@@ -37194,7 +37194,7 @@
         <v>6</v>
       </c>
       <c r="C11" s="7">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D11" s="7">
         <v>0</v>
@@ -37207,9 +37207,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H11" s="10" t="e">
+      <c r="H11" s="10">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="I11" s="10">
         <f t="shared" si="1"/>
@@ -37224,7 +37224,7 @@
         <v>6</v>
       </c>
       <c r="C12" s="7">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D12" s="7">
         <v>0</v>
@@ -37237,9 +37237,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H12" s="10" t="e">
+      <c r="H12" s="10">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="I12" s="10">
         <f t="shared" si="1"/>
@@ -37289,7 +37289,7 @@
       </c>
       <c r="C16" s="7">
         <f>SUM(C9:C14)</f>
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="D16" s="7">
         <f>SUM(D9:D14)</f>
@@ -37304,9 +37304,9 @@
         <f t="shared" ref="G16:H16" si="2">D16/B16</f>
         <v>0</v>
       </c>
-      <c r="H16" s="10" t="e">
+      <c r="H16" s="10">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="I16" s="10">
         <f t="shared" si="1"/>

</xml_diff>